<commit_message>
changes to plot functions
</commit_message>
<xml_diff>
--- a/examples/cond.xlsx
+++ b/examples/cond.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="26731"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="24332"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://ethz-my.sharepoint.com/personal/florinl_ethz_ch/Documents/Repositories/muf-bvar/Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\U80856195\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="8" documentId="13_ncr:1_{5AA1306C-24F5-4961-90B5-8621B8A8E65F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{93E26480-CAA6-4774-9EA0-F2C2017A5AE2}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{245476E3-3591-4554-B1A9-1CCACB594575}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2340" yWindow="2340" windowWidth="38700" windowHeight="15345" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1950" windowWidth="38700" windowHeight="15345" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Q" sheetId="2" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="8">
   <si>
     <t>w_1</t>
   </si>
@@ -85,7 +85,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="4">
     <border>
       <left/>
       <right/>
@@ -115,11 +115,20 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -134,6 +143,9 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -747,14 +759,14 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:D240"/>
+  <dimension ref="A1:E240"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="3" width="57.85546875" style="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
         <v>2</v>
       </c>
@@ -764,8 +776,11 @@
       <c r="D1" s="2" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E1" s="6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -778,8 +793,11 @@
       <c r="D2" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="3" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E2" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -792,8 +810,11 @@
       <c r="D3" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="4" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E3" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -806,8 +827,11 @@
       <c r="D4" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="5" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E4" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -820,8 +844,11 @@
       <c r="D5" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="6" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E5" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -834,8 +861,11 @@
       <c r="D6" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="7" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E6" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -848,8 +878,11 @@
       <c r="D7" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="8" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E7" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -862,8 +895,11 @@
       <c r="D8" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="9" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E8" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -876,8 +912,11 @@
       <c r="D9" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="10" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E9" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -890,8 +929,11 @@
       <c r="D10" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="11" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E10" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -904,8 +946,11 @@
       <c r="D11" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="12" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E11" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -918,8 +963,11 @@
       <c r="D12" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="13" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E12" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -932,8 +980,11 @@
       <c r="D13" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="14" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E13" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -946,8 +997,11 @@
       <c r="D14" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="15" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E14" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -960,8 +1014,11 @@
       <c r="D15" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="16" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E15" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -974,8 +1031,11 @@
       <c r="D16" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="17" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E16" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -988,8 +1048,11 @@
       <c r="D17" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="18" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E17" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -1002,8 +1065,11 @@
       <c r="D18" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="19" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E18" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -1016,8 +1082,11 @@
       <c r="D19" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="20" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E19" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -1030,8 +1099,11 @@
       <c r="D20" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="21" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E20" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -1044,8 +1116,11 @@
       <c r="D21" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="22" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E21" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -1058,8 +1133,11 @@
       <c r="D22" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="23" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E22" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -1072,8 +1150,11 @@
       <c r="D23" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="24" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E23" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -1086,8 +1167,11 @@
       <c r="D24" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="25" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E24" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -1100,26 +1184,29 @@
       <c r="D25" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="26" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E25" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3"/>
     </row>
-    <row r="27" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3"/>
     </row>
-    <row r="28" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3"/>
     </row>
-    <row r="29" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3"/>
     </row>
-    <row r="30" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3"/>
     </row>
-    <row r="31" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3"/>
     </row>
-    <row r="32" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3"/>
     </row>
     <row r="33" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
@@ -1756,14 +1843,14 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:E960"/>
+  <dimension ref="A1:I960"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="5" width="13.5703125" style="5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1776,8 +1863,20 @@
       <c r="E1" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F1" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>5</v>
+      </c>
+      <c r="I1" s="6" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="3">
         <v>1</v>
       </c>
@@ -1793,8 +1892,20 @@
       <c r="E2" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F2" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G2" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H2" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I2" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3">
         <v>2</v>
       </c>
@@ -1810,8 +1921,20 @@
       <c r="E3" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F3" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G3" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H3" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I3" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="3">
         <v>3</v>
       </c>
@@ -1827,8 +1950,20 @@
       <c r="E4" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F4" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G4" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H4" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I4" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="3">
         <v>4</v>
       </c>
@@ -1844,8 +1979,20 @@
       <c r="E5" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F5" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G5" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H5" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I5" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="3">
         <v>5</v>
       </c>
@@ -1861,8 +2008,20 @@
       <c r="E6" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F6" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G6" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H6" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I6" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="3">
         <v>6</v>
       </c>
@@ -1878,8 +2037,20 @@
       <c r="E7" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F7" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G7" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H7" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I7" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="3">
         <v>7</v>
       </c>
@@ -1895,8 +2066,20 @@
       <c r="E8" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F8" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G8" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H8" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I8" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="3">
         <v>8</v>
       </c>
@@ -1912,8 +2095,20 @@
       <c r="E9" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F9" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G9" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H9" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I9" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="3">
         <v>9</v>
       </c>
@@ -1929,8 +2124,20 @@
       <c r="E10" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F10" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G10" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H10" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I10" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3">
         <v>10</v>
       </c>
@@ -1946,8 +2153,20 @@
       <c r="E11" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F11" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G11" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H11" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I11" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="3">
         <v>11</v>
       </c>
@@ -1963,8 +2182,20 @@
       <c r="E12" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F12" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G12" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H12" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I12" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="3">
         <v>12</v>
       </c>
@@ -1980,8 +2211,20 @@
       <c r="E13" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F13" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G13" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H13" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I13" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="14" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="3">
         <v>13</v>
       </c>
@@ -1997,8 +2240,20 @@
       <c r="E14" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F14" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G14" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H14" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I14" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="15" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="3">
         <v>14</v>
       </c>
@@ -2014,8 +2269,20 @@
       <c r="E15" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F15" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G15" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H15" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I15" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="16" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="3">
         <v>15</v>
       </c>
@@ -2031,8 +2298,20 @@
       <c r="E16" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F16" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G16" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H16" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I16" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="3">
         <v>16</v>
       </c>
@@ -2048,8 +2327,20 @@
       <c r="E17" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F17" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G17" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H17" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I17" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="3">
         <v>17</v>
       </c>
@@ -2065,8 +2356,20 @@
       <c r="E18" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F18" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G18" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H18" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I18" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="3">
         <v>18</v>
       </c>
@@ -2082,8 +2385,20 @@
       <c r="E19" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F19" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G19" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H19" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I19" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="3">
         <v>19</v>
       </c>
@@ -2099,8 +2414,20 @@
       <c r="E20" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F20" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G20" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H20" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I20" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="3">
         <v>20</v>
       </c>
@@ -2116,8 +2443,20 @@
       <c r="E21" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F21" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G21" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H21" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I21" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="3">
         <v>21</v>
       </c>
@@ -2133,8 +2472,20 @@
       <c r="E22" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F22" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G22" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H22" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I22" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="3">
         <v>22</v>
       </c>
@@ -2150,8 +2501,20 @@
       <c r="E23" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F23" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G23" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H23" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I23" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="24" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="3">
         <v>23</v>
       </c>
@@ -2167,8 +2530,20 @@
       <c r="E24" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="25" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F24" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G24" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H24" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I24" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="25" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="3">
         <v>24</v>
       </c>
@@ -2184,8 +2559,20 @@
       <c r="E25" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="26" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F25" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G25" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H25" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I25" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="26" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="3">
         <v>25</v>
       </c>
@@ -2201,8 +2588,20 @@
       <c r="E26" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="27" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F26" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G26" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H26" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I26" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="3">
         <v>26</v>
       </c>
@@ -2218,8 +2617,20 @@
       <c r="E27" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="28" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F27" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G27" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H27" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I27" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="28" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="3">
         <v>27</v>
       </c>
@@ -2235,8 +2646,20 @@
       <c r="E28" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="29" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F28" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G28" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H28" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I28" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="29" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="3">
         <v>28</v>
       </c>
@@ -2252,8 +2675,20 @@
       <c r="E29" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="30" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F29" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G29" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H29" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I29" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="30" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="3">
         <v>29</v>
       </c>
@@ -2269,8 +2704,20 @@
       <c r="E30" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="31" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F30" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G30" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H30" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I30" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="31" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="3">
         <v>30</v>
       </c>
@@ -2286,8 +2733,20 @@
       <c r="E31" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="32" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F31" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G31" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H31" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I31" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="32" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="3">
         <v>31</v>
       </c>
@@ -2303,8 +2762,20 @@
       <c r="E32" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F32" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G32" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H32" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I32" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="33" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="3">
         <v>32</v>
       </c>
@@ -2320,8 +2791,20 @@
       <c r="E33" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="34" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F33" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G33" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H33" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I33" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="34" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="3">
         <v>33</v>
       </c>
@@ -2337,8 +2820,20 @@
       <c r="E34" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="35" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F34" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G34" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H34" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I34" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="35" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="3">
         <v>34</v>
       </c>
@@ -2354,8 +2849,20 @@
       <c r="E35" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="36" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F35" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G35" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H35" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I35" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="36" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="3">
         <v>35</v>
       </c>
@@ -2371,8 +2878,20 @@
       <c r="E36" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="37" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F36" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G36" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H36" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I36" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="37" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="3">
         <v>36</v>
       </c>
@@ -2388,8 +2907,20 @@
       <c r="E37" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="38" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F37" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G37" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H37" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I37" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="38" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="3">
         <v>37</v>
       </c>
@@ -2405,8 +2936,20 @@
       <c r="E38" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="39" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F38" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G38" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H38" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I38" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="39" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="3">
         <v>38</v>
       </c>
@@ -2422,8 +2965,20 @@
       <c r="E39" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="40" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F39" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G39" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H39" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I39" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="40" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="3">
         <v>39</v>
       </c>
@@ -2439,8 +2994,20 @@
       <c r="E40" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="41" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F40" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G40" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H40" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I40" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="41" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="3">
         <v>40</v>
       </c>
@@ -2456,8 +3023,20 @@
       <c r="E41" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="42" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F41" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G41" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H41" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I41" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="42" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="3">
         <v>41</v>
       </c>
@@ -2473,8 +3052,20 @@
       <c r="E42" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="43" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F42" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G42" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H42" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I42" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="43" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="3">
         <v>42</v>
       </c>
@@ -2490,8 +3081,20 @@
       <c r="E43" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="44" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F43" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G43" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H43" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I43" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="44" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="3">
         <v>43</v>
       </c>
@@ -2507,8 +3110,20 @@
       <c r="E44" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="45" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F44" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G44" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H44" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I44" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="45" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="3">
         <v>44</v>
       </c>
@@ -2524,8 +3139,20 @@
       <c r="E45" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="46" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F45" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G45" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H45" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I45" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="46" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="3">
         <v>45</v>
       </c>
@@ -2541,8 +3168,20 @@
       <c r="E46" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="47" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F46" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G46" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H46" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I46" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="47" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="3">
         <v>46</v>
       </c>
@@ -2558,8 +3197,20 @@
       <c r="E47" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="48" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F47" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G47" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H47" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I47" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="48" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="3">
         <v>47</v>
       </c>
@@ -2575,8 +3226,20 @@
       <c r="E48" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="49" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F48" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G48" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H48" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I48" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="49" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="3">
         <v>48</v>
       </c>
@@ -2592,8 +3255,20 @@
       <c r="E49" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="50" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F49" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G49" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H49" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I49" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="50" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="3">
         <v>49</v>
       </c>
@@ -2609,8 +3284,20 @@
       <c r="E50" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="51" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F50" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G50" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H50" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I50" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="51" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="3">
         <v>50</v>
       </c>
@@ -2626,8 +3313,20 @@
       <c r="E51" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="52" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F51" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G51" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H51" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I51" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="52" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="3">
         <v>51</v>
       </c>
@@ -2643,8 +3342,20 @@
       <c r="E52" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="53" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F52" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G52" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H52" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I52" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="53" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3">
         <v>52</v>
       </c>
@@ -2660,8 +3371,20 @@
       <c r="E53" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="54" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F53" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G53" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H53" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I53" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="54" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="3">
         <v>53</v>
       </c>
@@ -2677,8 +3400,20 @@
       <c r="E54" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="55" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F54" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G54" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H54" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I54" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="55" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3">
         <v>54</v>
       </c>
@@ -2694,8 +3429,20 @@
       <c r="E55" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="56" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F55" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G55" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H55" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I55" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="56" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3">
         <v>55</v>
       </c>
@@ -2711,8 +3458,20 @@
       <c r="E56" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="57" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F56" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G56" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H56" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I56" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="57" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3">
         <v>56</v>
       </c>
@@ -2728,8 +3487,20 @@
       <c r="E57" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="58" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F57" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G57" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H57" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I57" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="58" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3">
         <v>57</v>
       </c>
@@ -2745,8 +3516,20 @@
       <c r="E58" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="59" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F58" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G58" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H58" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I58" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="59" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3">
         <v>58</v>
       </c>
@@ -2762,8 +3545,20 @@
       <c r="E59" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="60" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F59" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G59" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H59" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I59" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="60" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3">
         <v>59</v>
       </c>
@@ -2779,8 +3574,20 @@
       <c r="E60" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="61" spans="1:5" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F60" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G60" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H60" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I60" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="61" spans="1:9" ht="19.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3">
         <v>60</v>
       </c>
@@ -2796,8 +3603,20 @@
       <c r="E61" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="62" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F61" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G61" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H61" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I61" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="62" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="3">
         <v>61</v>
       </c>
@@ -2813,8 +3632,20 @@
       <c r="E62" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="63" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F62" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G62" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H62" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I62" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="63" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="3">
         <v>62</v>
       </c>
@@ -2830,8 +3661,20 @@
       <c r="E63" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="64" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F63" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G63" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H63" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I63" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="64" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="3">
         <v>63</v>
       </c>
@@ -2847,8 +3690,20 @@
       <c r="E64" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="65" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F64" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G64" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H64" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I64" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="65" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3">
         <v>64</v>
       </c>
@@ -2864,8 +3719,20 @@
       <c r="E65" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="66" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F65" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G65" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H65" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I65" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="66" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="3">
         <v>65</v>
       </c>
@@ -2881,8 +3748,20 @@
       <c r="E66" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="67" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F66" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G66" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H66" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I66" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="67" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3">
         <v>66</v>
       </c>
@@ -2898,8 +3777,20 @@
       <c r="E67" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="68" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F67" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G67" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H67" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I67" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="3">
         <v>67</v>
       </c>
@@ -2915,8 +3806,20 @@
       <c r="E68" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="69" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F68" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G68" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H68" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I68" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="3">
         <v>68</v>
       </c>
@@ -2932,8 +3835,20 @@
       <c r="E69" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="70" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F69" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G69" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H69" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I69" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="3">
         <v>69</v>
       </c>
@@ -2949,8 +3864,20 @@
       <c r="E70" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="71" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F70" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G70" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H70" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I70" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="3">
         <v>70</v>
       </c>
@@ -2966,8 +3893,20 @@
       <c r="E71" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="72" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F71" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G71" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H71" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I71" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="3">
         <v>71</v>
       </c>
@@ -2983,8 +3922,20 @@
       <c r="E72" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="73" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F72" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G72" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H72" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I72" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="73" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="3">
         <v>72</v>
       </c>
@@ -3000,8 +3951,20 @@
       <c r="E73" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="74" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F73" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G73" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H73" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I73" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="3">
         <v>73</v>
       </c>
@@ -3017,8 +3980,20 @@
       <c r="E74" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="75" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F74" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G74" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H74" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I74" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="3">
         <v>74</v>
       </c>
@@ -3034,8 +4009,20 @@
       <c r="E75" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="76" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F75" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G75" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H75" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I75" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="3">
         <v>75</v>
       </c>
@@ -3051,8 +4038,20 @@
       <c r="E76" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="77" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F76" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G76" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H76" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I76" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="3">
         <v>76</v>
       </c>
@@ -3068,8 +4067,20 @@
       <c r="E77" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="78" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F77" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G77" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H77" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I77" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="3">
         <v>77</v>
       </c>
@@ -3085,8 +4096,20 @@
       <c r="E78" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="79" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F78" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G78" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H78" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I78" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="3">
         <v>78</v>
       </c>
@@ -3102,8 +4125,20 @@
       <c r="E79" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="80" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F79" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G79" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H79" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I79" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="80" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="3">
         <v>79</v>
       </c>
@@ -3119,8 +4154,20 @@
       <c r="E80" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="81" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F80" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G80" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H80" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I80" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="81" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="3">
         <v>80</v>
       </c>
@@ -3136,8 +4183,20 @@
       <c r="E81" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="82" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F81" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G81" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H81" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I81" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="82" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="3">
         <v>81</v>
       </c>
@@ -3153,8 +4212,20 @@
       <c r="E82" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="83" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F82" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G82" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H82" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I82" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="83" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="3">
         <v>82</v>
       </c>
@@ -3170,8 +4241,20 @@
       <c r="E83" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="84" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F83" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G83" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H83" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I83" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="84" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="3">
         <v>83</v>
       </c>
@@ -3187,8 +4270,20 @@
       <c r="E84" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="85" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F84" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G84" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H84" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I84" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="85" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="3">
         <v>84</v>
       </c>
@@ -3204,8 +4299,20 @@
       <c r="E85" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="86" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F85" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G85" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H85" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I85" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="86" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="3">
         <v>85</v>
       </c>
@@ -3221,8 +4328,20 @@
       <c r="E86" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="87" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F86" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G86" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H86" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I86" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="87" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="3">
         <v>86</v>
       </c>
@@ -3238,8 +4357,20 @@
       <c r="E87" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="88" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F87" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G87" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H87" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I87" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="88" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="3">
         <v>87</v>
       </c>
@@ -3255,8 +4386,20 @@
       <c r="E88" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="89" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F88" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G88" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H88" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I88" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="89" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="3">
         <v>88</v>
       </c>
@@ -3272,8 +4415,20 @@
       <c r="E89" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="90" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F89" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G89" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H89" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I89" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="90" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="3">
         <v>89</v>
       </c>
@@ -3289,8 +4444,20 @@
       <c r="E90" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="91" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F90" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G90" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H90" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I90" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="91" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="3">
         <v>90</v>
       </c>
@@ -3306,8 +4473,20 @@
       <c r="E91" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="92" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F91" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G91" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H91" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I91" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="92" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="3">
         <v>91</v>
       </c>
@@ -3323,8 +4502,20 @@
       <c r="E92" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="93" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F92" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G92" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H92" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I92" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="93" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="3">
         <v>92</v>
       </c>
@@ -3340,8 +4531,20 @@
       <c r="E93" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="94" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F93" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G93" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H93" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I93" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="94" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="3">
         <v>93</v>
       </c>
@@ -3357,8 +4560,20 @@
       <c r="E94" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="95" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F94" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G94" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H94" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I94" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="95" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="3">
         <v>94</v>
       </c>
@@ -3374,8 +4589,20 @@
       <c r="E95" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="96" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F95" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G95" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H95" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I95" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="96" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="3">
         <v>95</v>
       </c>
@@ -3391,8 +4618,20 @@
       <c r="E96" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="97" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F96" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G96" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H96" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I96" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="97" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="3">
         <v>96</v>
       </c>
@@ -3408,50 +4647,77 @@
       <c r="E97" s="4">
         <v>9.8899999999999999E+42</v>
       </c>
-    </row>
-    <row r="98" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="F97" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="G97" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="H97" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+      <c r="I97" s="4">
+        <v>9.8899999999999999E+42</v>
+      </c>
+    </row>
+    <row r="98" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="3"/>
-    </row>
-    <row r="99" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E98" s="4"/>
+      <c r="F98" s="4"/>
+      <c r="G98" s="4"/>
+      <c r="H98" s="4"/>
+      <c r="I98" s="4"/>
+    </row>
+    <row r="99" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="3"/>
-    </row>
-    <row r="100" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E99" s="4"/>
+      <c r="F99" s="4"/>
+      <c r="G99" s="4"/>
+      <c r="H99" s="4"/>
+      <c r="I99" s="4"/>
+    </row>
+    <row r="100" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="3"/>
-    </row>
-    <row r="101" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="E100" s="4"/>
+      <c r="F100" s="4"/>
+      <c r="G100" s="4"/>
+      <c r="H100" s="4"/>
+      <c r="I100" s="4"/>
+    </row>
+    <row r="101" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="3"/>
     </row>
-    <row r="102" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A102" s="3"/>
     </row>
-    <row r="103" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A103" s="3"/>
     </row>
-    <row r="104" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A104" s="3"/>
     </row>
-    <row r="105" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A105" s="3"/>
     </row>
-    <row r="106" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A106" s="3"/>
     </row>
-    <row r="107" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A107" s="3"/>
     </row>
-    <row r="108" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A108" s="3"/>
     </row>
-    <row r="109" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A109" s="3"/>
     </row>
-    <row r="110" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A110" s="3"/>
     </row>
-    <row r="111" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A111" s="3"/>
     </row>
-    <row r="112" spans="1:5" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A112" s="3"/>
     </row>
     <row r="113" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">

</xml_diff>